<commit_message>
Update Visit type 'Pre-Treatment' and 'First Dose' or 'FD' value
</commit_message>
<xml_diff>
--- a/inst/extdata/example_visitcode.xlsx
+++ b/inst/extdata/example_visitcode.xlsx
@@ -4,12 +4,13 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6390"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6390" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="QL1706-303" sheetId="5" r:id="rId1"/>
-    <sheet name="QL0911-302" sheetId="4" r:id="rId2"/>
-    <sheet name="QLG1079-303" sheetId="3" r:id="rId3"/>
+    <sheet name="QLS31905-301" sheetId="6" r:id="rId2"/>
+    <sheet name="QL0911-302" sheetId="4" r:id="rId3"/>
+    <sheet name="QLG1079-303" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="374">
   <si>
     <t>随访期</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -531,13 +532,711 @@
   </si>
   <si>
     <t>VISITDAY</t>
+  </si>
+  <si>
+    <t>VISITNUM</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>WP</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>VISITDAY</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>筛选期</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>-28d</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>筛选期1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>预激访视</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>C1D1</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>治疗期1</t>
+  </si>
+  <si>
+    <t>C1D8</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>C2D1</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>C2D8</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>C3D1</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>C3D8</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>±2d</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>C4D1</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>C4D8</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>C5D1</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>C5D8</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>C6D1</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>C6D8</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>C7D1</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>±3d</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>C7D8</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>C8D1</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>C8D8</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>C9D1</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>C9D8</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>C10D1</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>C10D8</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>C11D1</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>C11D8</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>C12D1</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>C12D8</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>C13D1</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>C13D8</t>
+  </si>
+  <si>
+    <t>29</t>
+  </si>
+  <si>
+    <t>C14D1</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>C14D8</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>C15D1</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
+    <t>C15D8</t>
+  </si>
+  <si>
+    <t>33</t>
+  </si>
+  <si>
+    <t>C16D1</t>
+  </si>
+  <si>
+    <t>34</t>
+  </si>
+  <si>
+    <t>C16D8</t>
+  </si>
+  <si>
+    <t>35</t>
+  </si>
+  <si>
+    <t>C17D1</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>C17D8</t>
+  </si>
+  <si>
+    <t>37</t>
+  </si>
+  <si>
+    <t>C18D1</t>
+  </si>
+  <si>
+    <t>38</t>
+  </si>
+  <si>
+    <t>C18D8</t>
+  </si>
+  <si>
+    <t>39</t>
+  </si>
+  <si>
+    <t>C19D1</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>C19D8</t>
+  </si>
+  <si>
+    <t>41</t>
+  </si>
+  <si>
+    <t>C20D1</t>
+  </si>
+  <si>
+    <t>42</t>
+  </si>
+  <si>
+    <t>C20D8</t>
+  </si>
+  <si>
+    <t>43</t>
+  </si>
+  <si>
+    <t>C21D1</t>
+  </si>
+  <si>
+    <t>44</t>
+  </si>
+  <si>
+    <t>C21D8</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>C22D1</t>
+  </si>
+  <si>
+    <t>46</t>
+  </si>
+  <si>
+    <t>C22D8</t>
+  </si>
+  <si>
+    <t>47</t>
+  </si>
+  <si>
+    <t>C23D1</t>
+  </si>
+  <si>
+    <t>48</t>
+  </si>
+  <si>
+    <t>C23D8</t>
+  </si>
+  <si>
+    <t>49</t>
+  </si>
+  <si>
+    <t>C24D1</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>C24D8</t>
+  </si>
+  <si>
+    <t>51</t>
+  </si>
+  <si>
+    <t>C25D1</t>
+  </si>
+  <si>
+    <t>52</t>
+  </si>
+  <si>
+    <t>C25D8</t>
+  </si>
+  <si>
+    <t>53</t>
+  </si>
+  <si>
+    <t>C26D1</t>
+  </si>
+  <si>
+    <t>54</t>
+  </si>
+  <si>
+    <t>C26D8</t>
+  </si>
+  <si>
+    <t>55</t>
+  </si>
+  <si>
+    <t>C27D1</t>
+  </si>
+  <si>
+    <t>56</t>
+  </si>
+  <si>
+    <t>C27D8</t>
+  </si>
+  <si>
+    <t>57</t>
+  </si>
+  <si>
+    <t>C28D1</t>
+  </si>
+  <si>
+    <t>58</t>
+  </si>
+  <si>
+    <t>C28D8</t>
+  </si>
+  <si>
+    <t>59</t>
+  </si>
+  <si>
+    <t>C29D1</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>C29D8</t>
+  </si>
+  <si>
+    <t>61</t>
+  </si>
+  <si>
+    <t>C30D1</t>
+  </si>
+  <si>
+    <t>62</t>
+  </si>
+  <si>
+    <t>C30D8</t>
+  </si>
+  <si>
+    <t>63</t>
+  </si>
+  <si>
+    <t>C31D1</t>
+  </si>
+  <si>
+    <t>64</t>
+  </si>
+  <si>
+    <t>C31D8</t>
+  </si>
+  <si>
+    <t>65</t>
+  </si>
+  <si>
+    <t>C32D1</t>
+  </si>
+  <si>
+    <t>66</t>
+  </si>
+  <si>
+    <t>C32D8</t>
+  </si>
+  <si>
+    <t>67</t>
+  </si>
+  <si>
+    <t>C33D1</t>
+  </si>
+  <si>
+    <t>68</t>
+  </si>
+  <si>
+    <t>C33D8</t>
+  </si>
+  <si>
+    <t>69</t>
+  </si>
+  <si>
+    <t>C34D1</t>
+  </si>
+  <si>
+    <t>70</t>
+  </si>
+  <si>
+    <t>C34D8</t>
+  </si>
+  <si>
+    <t>71</t>
+  </si>
+  <si>
+    <t>C35D1</t>
+  </si>
+  <si>
+    <t>72</t>
+  </si>
+  <si>
+    <t>C35D8</t>
+  </si>
+  <si>
+    <t>73</t>
+  </si>
+  <si>
+    <t>C36D1</t>
+  </si>
+  <si>
+    <t>74</t>
+  </si>
+  <si>
+    <t>治疗期36</t>
+  </si>
+  <si>
+    <t>C36D8</t>
+  </si>
+  <si>
+    <t>75</t>
+  </si>
+  <si>
+    <t>C37D1</t>
+  </si>
+  <si>
+    <t>76</t>
+  </si>
+  <si>
+    <t>治疗期37</t>
+  </si>
+  <si>
+    <t>C37D8</t>
+  </si>
+  <si>
+    <t>77</t>
+  </si>
+  <si>
+    <t>C38D1</t>
+  </si>
+  <si>
+    <t>78</t>
+  </si>
+  <si>
+    <t>治疗期38</t>
+  </si>
+  <si>
+    <t>C38D8</t>
+  </si>
+  <si>
+    <t>79</t>
+  </si>
+  <si>
+    <t>C39D1</t>
+  </si>
+  <si>
+    <t>80</t>
+  </si>
+  <si>
+    <t>治疗期39</t>
+  </si>
+  <si>
+    <t>C39D8</t>
+  </si>
+  <si>
+    <t>81</t>
+  </si>
+  <si>
+    <t>C40D1</t>
+  </si>
+  <si>
+    <t>82</t>
+  </si>
+  <si>
+    <t>治疗期40</t>
+  </si>
+  <si>
+    <t>C40D8</t>
+  </si>
+  <si>
+    <t>83</t>
+  </si>
+  <si>
+    <t>C41D1</t>
+  </si>
+  <si>
+    <t>84</t>
+  </si>
+  <si>
+    <t>治疗期41</t>
+  </si>
+  <si>
+    <t>C41D8</t>
+  </si>
+  <si>
+    <t>85</t>
+  </si>
+  <si>
+    <t>C42D1</t>
+  </si>
+  <si>
+    <t>86</t>
+  </si>
+  <si>
+    <t>治疗期42</t>
+  </si>
+  <si>
+    <t>C42D8</t>
+  </si>
+  <si>
+    <t>87</t>
+  </si>
+  <si>
+    <t>C43D1</t>
+  </si>
+  <si>
+    <t>88</t>
+  </si>
+  <si>
+    <t>治疗期43</t>
+  </si>
+  <si>
+    <t>C43D8</t>
+  </si>
+  <si>
+    <t>89</t>
+  </si>
+  <si>
+    <t>C44D1</t>
+  </si>
+  <si>
+    <t>90</t>
+  </si>
+  <si>
+    <t>治疗期44</t>
+  </si>
+  <si>
+    <t>C44D8</t>
+  </si>
+  <si>
+    <t>91</t>
+  </si>
+  <si>
+    <t>C45D1</t>
+  </si>
+  <si>
+    <t>92</t>
+  </si>
+  <si>
+    <t>治疗期45</t>
+  </si>
+  <si>
+    <t>C45D8</t>
+  </si>
+  <si>
+    <t>93</t>
+  </si>
+  <si>
+    <t>治疗结束/提前退出</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+7d </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+      </rPr>
+      <t>治疗结束</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>EOT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>安全性随访-末次用药30天</t>
+  </si>
+  <si>
+    <t>142</t>
+  </si>
+  <si>
+    <t>安全性随访-末次用药60天</t>
+  </si>
+  <si>
+    <t>143</t>
+  </si>
+  <si>
+    <t>±7d</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>随访期</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LD+60</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>安全性随访-末次用药90天</t>
+  </si>
+  <si>
+    <t>144</t>
+  </si>
+  <si>
+    <t>146</t>
+  </si>
+  <si>
+    <t>研究结束</t>
+  </si>
+  <si>
+    <t>147</t>
+  </si>
+  <si>
+    <t>研究结束</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>预治疗期</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>FD</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -554,6 +1253,25 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <family val="3"/>
       <charset val="134"/>
@@ -579,7 +1297,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -590,6 +1308,14 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -871,13 +1597,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E44"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="23.6640625" customWidth="1"/>
     <col min="2" max="2" width="18.9140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="14.5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="14.5">
       <c r="A1" s="4" t="s">
         <v>145</v>
       </c>
@@ -894,7 +1620,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
         <v>56</v>
       </c>
@@ -908,7 +1634,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5">
       <c r="A3" s="1" t="s">
         <v>57</v>
       </c>
@@ -922,7 +1648,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
         <v>58</v>
       </c>
@@ -939,7 +1665,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5">
       <c r="A5" s="1" t="s">
         <v>59</v>
       </c>
@@ -956,7 +1682,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5">
       <c r="A6" s="1" t="s">
         <v>60</v>
       </c>
@@ -973,7 +1699,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5">
       <c r="A7" s="1" t="s">
         <v>61</v>
       </c>
@@ -990,7 +1716,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5">
       <c r="A8" s="1" t="s">
         <v>62</v>
       </c>
@@ -1007,7 +1733,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5">
       <c r="A9" s="1" t="s">
         <v>63</v>
       </c>
@@ -1024,7 +1750,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5">
       <c r="A10" s="1" t="s">
         <v>64</v>
       </c>
@@ -1041,7 +1767,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5">
       <c r="A11" s="1" t="s">
         <v>65</v>
       </c>
@@ -1058,7 +1784,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5">
       <c r="A12" s="1" t="s">
         <v>66</v>
       </c>
@@ -1075,7 +1801,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5">
       <c r="A13" s="1" t="s">
         <v>67</v>
       </c>
@@ -1092,7 +1818,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5">
       <c r="A14" s="1" t="s">
         <v>68</v>
       </c>
@@ -1109,7 +1835,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5">
       <c r="A15" s="1" t="s">
         <v>69</v>
       </c>
@@ -1126,7 +1852,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5">
       <c r="A16" s="1" t="s">
         <v>70</v>
       </c>
@@ -1143,7 +1869,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5">
       <c r="A17" s="1" t="s">
         <v>71</v>
       </c>
@@ -1160,7 +1886,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5">
       <c r="A18" s="1" t="s">
         <v>72</v>
       </c>
@@ -1177,7 +1903,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5">
       <c r="A19" s="1" t="s">
         <v>73</v>
       </c>
@@ -1194,7 +1920,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5">
       <c r="A20" s="1" t="s">
         <v>74</v>
       </c>
@@ -1211,7 +1937,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5">
       <c r="A21" s="1" t="s">
         <v>75</v>
       </c>
@@ -1228,7 +1954,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5">
       <c r="A22" s="1" t="s">
         <v>76</v>
       </c>
@@ -1245,7 +1971,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5">
       <c r="A23" s="1" t="s">
         <v>77</v>
       </c>
@@ -1262,7 +1988,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5">
       <c r="A24" s="1" t="s">
         <v>78</v>
       </c>
@@ -1279,7 +2005,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5">
       <c r="A25" s="1" t="s">
         <v>79</v>
       </c>
@@ -1296,7 +2022,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5">
       <c r="A26" s="1" t="s">
         <v>80</v>
       </c>
@@ -1313,7 +2039,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5">
       <c r="A27" s="1" t="s">
         <v>81</v>
       </c>
@@ -1330,7 +2056,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5">
       <c r="A28" s="1" t="s">
         <v>82</v>
       </c>
@@ -1347,7 +2073,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5">
       <c r="A29" s="1" t="s">
         <v>83</v>
       </c>
@@ -1364,7 +2090,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5">
       <c r="A30" s="1" t="s">
         <v>84</v>
       </c>
@@ -1381,7 +2107,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5">
       <c r="A31" s="1" t="s">
         <v>85</v>
       </c>
@@ -1398,7 +2124,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5">
       <c r="A32" s="1" t="s">
         <v>86</v>
       </c>
@@ -1415,7 +2141,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5">
       <c r="A33" s="1" t="s">
         <v>87</v>
       </c>
@@ -1432,7 +2158,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5">
       <c r="A34" s="1" t="s">
         <v>88</v>
       </c>
@@ -1449,7 +2175,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5">
       <c r="A35" s="1" t="s">
         <v>89</v>
       </c>
@@ -1466,7 +2192,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5">
       <c r="A36" s="1" t="s">
         <v>90</v>
       </c>
@@ -1483,7 +2209,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5">
       <c r="A37" s="1" t="s">
         <v>91</v>
       </c>
@@ -1500,7 +2226,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5">
       <c r="A38" s="1" t="s">
         <v>92</v>
       </c>
@@ -1517,7 +2243,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5">
       <c r="A39" s="1" t="s">
         <v>10</v>
       </c>
@@ -1534,7 +2260,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5">
       <c r="A40" s="1" t="s">
         <v>93</v>
       </c>
@@ -1551,7 +2277,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5">
       <c r="A41" s="1" t="s">
         <v>94</v>
       </c>
@@ -1568,7 +2294,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5">
       <c r="A42" s="1" t="s">
         <v>95</v>
       </c>
@@ -1585,7 +2311,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5">
       <c r="A43" s="1" t="s">
         <v>96</v>
       </c>
@@ -1602,7 +2328,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5">
       <c r="A44" s="1" t="s">
         <v>12</v>
       </c>
@@ -1627,334 +2353,1688 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E20"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="21.6640625" customWidth="1"/>
-    <col min="2" max="2" width="11.4140625" customWidth="1"/>
-    <col min="3" max="3" width="9.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:E99"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <sheetData>
-    <row r="1" spans="1:5" ht="14.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
         <v>140</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D1" s="5" t="s">
+      <c r="B1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="D1" t="s">
         <v>143</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" s="1">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+        <v>153</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" s="1">
-        <v>2</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+        <v>157</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="E3" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" s="1">
-        <v>6</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4" t="s">
-        <v>28</v>
+        <v>161</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>163</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5">
       <c r="A5" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5" s="1">
-        <v>7</v>
-      </c>
-      <c r="C5" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" t="s">
-        <v>28</v>
+        <v>164</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>163</v>
       </c>
       <c r="E5">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5">
       <c r="A6" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B6" s="1">
-        <v>8</v>
-      </c>
-      <c r="C6" t="s">
-        <v>30</v>
-      </c>
-      <c r="D6" t="s">
-        <v>28</v>
+        <v>166</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>100</v>
       </c>
       <c r="E6">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
       <c r="A7" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B7" s="1">
-        <v>9</v>
-      </c>
-      <c r="C7" t="s">
-        <v>30</v>
-      </c>
-      <c r="D7" t="s">
-        <v>28</v>
+        <v>168</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>100</v>
       </c>
       <c r="E7">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
       <c r="A8" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B8" s="1">
-        <v>10</v>
-      </c>
-      <c r="C8" t="s">
+        <v>170</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="E9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="E11">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="C13" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D8" t="s">
-        <v>35</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B9" s="1">
-        <v>11</v>
-      </c>
-      <c r="C9" t="s">
-        <v>30</v>
-      </c>
-      <c r="D9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E9">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B10" s="1">
-        <v>12</v>
-      </c>
-      <c r="C10" t="s">
-        <v>30</v>
-      </c>
-      <c r="D10" t="s">
-        <v>35</v>
-      </c>
-      <c r="E10">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" s="1">
-        <v>13</v>
-      </c>
-      <c r="C11" t="s">
-        <v>30</v>
-      </c>
-      <c r="D11" t="s">
-        <v>35</v>
-      </c>
-      <c r="E11">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" s="1">
-        <v>14</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="D13" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="E13">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="E15">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="E17">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="E19">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="C21" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D12" t="s">
-        <v>40</v>
-      </c>
-      <c r="E12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B13" s="1">
-        <v>15</v>
-      </c>
-      <c r="C13" t="s">
-        <v>30</v>
-      </c>
-      <c r="D13" t="s">
-        <v>40</v>
-      </c>
-      <c r="E13">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B14" s="1">
-        <v>16</v>
-      </c>
-      <c r="C14" t="s">
-        <v>30</v>
-      </c>
-      <c r="D14" t="s">
-        <v>40</v>
-      </c>
-      <c r="E14">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B15" s="1">
+      <c r="D21" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="E21">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="E23">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="E25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="E27">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="E29">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="E30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="E31">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="E32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="E33">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E35">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
+      <c r="A36" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="E36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="E37">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
+      <c r="A38" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="E38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5">
+      <c r="A39" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D39" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="E39">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
+      <c r="A40" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D40" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="E40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="A41" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D41" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="E41">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5">
+      <c r="A42" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D42" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="E42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
+      <c r="A43" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D43" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="E43">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5">
+      <c r="A44" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="D44" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="E44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5">
+      <c r="A45" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D45" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="E45">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
+      <c r="A46" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="D46" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="E46">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5">
+      <c r="A47" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D47" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="E47">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5">
+      <c r="A48" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="D48" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="E48">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5">
+      <c r="A49" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D49" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="E49">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5">
+      <c r="A50" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D50" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="E50">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5">
+      <c r="A51" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D51" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="E51">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5">
+      <c r="A52" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="D52" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="E52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5">
+      <c r="A53" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D53" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="E53">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5">
+      <c r="A54" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D54" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="E54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5">
+      <c r="A55" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D55" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="E55">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5">
+      <c r="A56" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D56" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="E56">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5">
+      <c r="A57" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D57" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="E57">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5">
+      <c r="A58" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="D58" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="E58">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5">
+      <c r="A59" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D59" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="E59">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5">
+      <c r="A60" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D60" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="E60">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5">
+      <c r="A61" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D61" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="E61">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5">
+      <c r="A62" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D62" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="E62">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5">
+      <c r="A63" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D63" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="E63">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5">
+      <c r="A64" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D64" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E64">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5">
+      <c r="A65" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D65" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E65">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5">
+      <c r="A66" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D66" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="E66">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5">
+      <c r="A67" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D67" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="E67">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5">
+      <c r="A68" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="D68" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="E68">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5">
+      <c r="A69" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D69" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="E69">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5">
+      <c r="A70" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D70" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="E70">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5">
+      <c r="A71" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D71" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="E71">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5">
+      <c r="A72" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D72" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="E72">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5">
+      <c r="A73" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D73" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="E73">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5">
+      <c r="A74" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="D74" s="8" t="s">
+        <v>306</v>
+      </c>
+      <c r="E74">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5">
+      <c r="A75" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D75" s="8" t="s">
+        <v>306</v>
+      </c>
+      <c r="E75">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5">
+      <c r="A76" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D76" s="8" t="s">
+        <v>311</v>
+      </c>
+      <c r="E76">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5">
+      <c r="A77" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D77" s="8" t="s">
+        <v>311</v>
+      </c>
+      <c r="E77">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5">
+      <c r="A78" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D78" s="8" t="s">
+        <v>316</v>
+      </c>
+      <c r="E78">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5">
+      <c r="A79" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D79" s="8" t="s">
+        <v>316</v>
+      </c>
+      <c r="E79">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5">
+      <c r="A80" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D80" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="E80">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5">
+      <c r="A81" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D81" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="E81">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5">
+      <c r="A82" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D82" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="E82">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5">
+      <c r="A83" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D83" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="E83">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5">
+      <c r="A84" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="D84" s="8" t="s">
+        <v>331</v>
+      </c>
+      <c r="E84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5">
+      <c r="A85" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="C85" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D85" s="8" t="s">
+        <v>331</v>
+      </c>
+      <c r="E85">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5">
+      <c r="A86" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="C86" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D86" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="E86">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5">
+      <c r="A87" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C87" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D87" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="E87">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5">
+      <c r="A88" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="C88" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D88" s="8" t="s">
+        <v>341</v>
+      </c>
+      <c r="E88">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5">
+      <c r="A89" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="C89" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D89" s="8" t="s">
+        <v>341</v>
+      </c>
+      <c r="E89">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5">
+      <c r="A90" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="C90" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D90" s="8" t="s">
+        <v>346</v>
+      </c>
+      <c r="E90">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5">
+      <c r="A91" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="C91" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D91" s="8" t="s">
+        <v>346</v>
+      </c>
+      <c r="E91">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5">
+      <c r="A92" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="D92" s="8" t="s">
+        <v>351</v>
+      </c>
+      <c r="E92">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5">
+      <c r="A93" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="C93" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D93" s="8" t="s">
+        <v>351</v>
+      </c>
+      <c r="E93">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5">
+      <c r="A94" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="C94" s="7" t="s">
+        <v>356</v>
+      </c>
+      <c r="D94" s="8" t="s">
+        <v>357</v>
+      </c>
+      <c r="E94" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5">
+      <c r="A95" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="C95" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D95" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C15" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" t="s">
-        <v>44</v>
-      </c>
-      <c r="E15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B16" s="1">
-        <v>18</v>
-      </c>
-      <c r="C16" t="s">
-        <v>30</v>
-      </c>
-      <c r="D16" t="s">
-        <v>44</v>
-      </c>
-      <c r="E16">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B17" s="1">
-        <v>19</v>
-      </c>
-      <c r="C17" t="s">
-        <v>30</v>
-      </c>
-      <c r="D17" t="s">
-        <v>44</v>
-      </c>
-      <c r="E17">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B18" s="1">
-        <v>20</v>
-      </c>
-      <c r="C18" t="s">
-        <v>48</v>
-      </c>
-      <c r="D18" t="s">
-        <v>49</v>
-      </c>
-      <c r="E18" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B19" s="1">
-        <v>21</v>
-      </c>
-      <c r="C19" t="s">
-        <v>34</v>
-      </c>
-      <c r="D19" t="s">
-        <v>52</v>
-      </c>
-      <c r="E19" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
+      <c r="E95" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5">
+      <c r="A96" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="C96" s="6" t="s">
+        <v>363</v>
+      </c>
+      <c r="D96" s="8" t="s">
+        <v>364</v>
+      </c>
+      <c r="E96" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5">
+      <c r="A97" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="C97" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D97" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E97" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5">
+      <c r="A98" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="C98" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D98" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E98" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5">
+      <c r="A99" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="C99" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="D99" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="E99" t="s">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -1964,14 +4044,351 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr defaultRowHeight="14"/>
+  <cols>
+    <col min="1" max="1" width="21.6640625" customWidth="1"/>
+    <col min="2" max="2" width="11.4140625" customWidth="1"/>
+    <col min="3" max="3" width="9.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="14.5">
+      <c r="A1" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="1">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="1">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="1">
+        <v>6</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="1">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="1">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="1">
+        <v>9</v>
+      </c>
+      <c r="C7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="1">
+        <v>10</v>
+      </c>
+      <c r="C8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" s="1">
+        <v>11</v>
+      </c>
+      <c r="C9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10" s="1">
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" t="s">
+        <v>35</v>
+      </c>
+      <c r="E10">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="1">
+        <v>13</v>
+      </c>
+      <c r="C11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" t="s">
+        <v>35</v>
+      </c>
+      <c r="E11">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="1">
+        <v>14</v>
+      </c>
+      <c r="C12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="1">
+        <v>15</v>
+      </c>
+      <c r="C13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" t="s">
+        <v>40</v>
+      </c>
+      <c r="E13">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="1">
+        <v>16</v>
+      </c>
+      <c r="C14" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" t="s">
+        <v>40</v>
+      </c>
+      <c r="E14">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="1">
+        <v>17</v>
+      </c>
+      <c r="C15" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" t="s">
+        <v>44</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" s="1">
+        <v>18</v>
+      </c>
+      <c r="C16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D16" t="s">
+        <v>44</v>
+      </c>
+      <c r="E16">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B17" s="1">
+        <v>19</v>
+      </c>
+      <c r="C17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D17" t="s">
+        <v>44</v>
+      </c>
+      <c r="E17">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="1">
+        <v>20</v>
+      </c>
+      <c r="C18" t="s">
+        <v>48</v>
+      </c>
+      <c r="D18" t="s">
+        <v>49</v>
+      </c>
+      <c r="E18" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" s="1">
+        <v>21</v>
+      </c>
+      <c r="C19" t="s">
+        <v>34</v>
+      </c>
+      <c r="D19" t="s">
+        <v>52</v>
+      </c>
+      <c r="E19" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="22.58203125" customWidth="1"/>
     <col min="2" max="2" width="15.08203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="14.5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="14.5">
       <c r="A1" s="4" t="s">
         <v>145</v>
       </c>
@@ -1988,7 +4405,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -2002,7 +4419,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -2019,7 +4436,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
         <v>54</v>
       </c>
@@ -2036,7 +4453,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -2053,7 +4470,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -2070,7 +4487,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
@@ -2087,7 +4504,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -2104,7 +4521,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5">
       <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
@@ -2121,7 +4538,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -2138,7 +4555,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5">
       <c r="A11" s="1" t="s">
         <v>11</v>
       </c>
@@ -2155,7 +4572,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5">
       <c r="A12" s="1" t="s">
         <v>12</v>
       </c>

</xml_diff>

<commit_message>
Update example excel file
</commit_message>
<xml_diff>
--- a/inst/extdata/example_visitcode.xlsx
+++ b/inst/extdata/example_visitcode.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6390" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6396" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="QL1706-303" sheetId="5" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="378">
   <si>
     <t>随访期</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1229,6 +1229,22 @@
   </si>
   <si>
     <t>FD</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>纠正治疗期_D1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>FD</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>纠正治疗期_D2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>纠正治疗期_D3</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1297,7 +1313,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1315,6 +1331,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1597,13 +1616,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E44"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="23.6640625" customWidth="1"/>
-    <col min="2" max="2" width="18.9140625" customWidth="1"/>
+    <col min="2" max="2" width="18.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="14.5">
+    <row r="1" spans="1:5" ht="14.4">
       <c r="A1" s="4" t="s">
         <v>145</v>
       </c>
@@ -2354,7 +2373,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E99"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
@@ -4044,15 +4063,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E20"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <dimension ref="A1:E23"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="21.6640625" customWidth="1"/>
-    <col min="2" max="2" width="11.4140625" customWidth="1"/>
-    <col min="3" max="3" width="9.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.44140625" customWidth="1"/>
+    <col min="3" max="3" width="9.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="14.5">
+    <row r="1" spans="1:5" ht="14.4">
       <c r="A1" s="4" t="s">
         <v>140</v>
       </c>
@@ -4098,204 +4117,204 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1" t="s">
-        <v>27</v>
+      <c r="A4" s="10" t="s">
+        <v>374</v>
       </c>
       <c r="B4" s="1">
-        <v>6</v>
-      </c>
-      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2">
         <v>0</v>
       </c>
-      <c r="D4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
+      <c r="D4" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="E4" t="s">
+        <v>375</v>
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1" t="s">
-        <v>29</v>
+      <c r="A5" s="10" t="s">
+        <v>376</v>
       </c>
       <c r="B5" s="1">
-        <v>7</v>
-      </c>
-      <c r="C5" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" t="s">
-        <v>28</v>
+        <v>4</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>372</v>
       </c>
       <c r="E5">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1" t="s">
-        <v>31</v>
+      <c r="A6" s="10" t="s">
+        <v>377</v>
       </c>
       <c r="B6" s="1">
-        <v>8</v>
-      </c>
-      <c r="C6" t="s">
-        <v>30</v>
-      </c>
-      <c r="D6" t="s">
-        <v>28</v>
+        <v>5</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>372</v>
       </c>
       <c r="E6">
-        <v>15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B7" s="1">
-        <v>9</v>
-      </c>
-      <c r="C7" t="s">
-        <v>30</v>
+        <v>6</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
       </c>
       <c r="D7" t="s">
         <v>28</v>
       </c>
       <c r="E7">
-        <v>21</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B8" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D8" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="E8">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="1" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B9" s="1">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C9" t="s">
         <v>30</v>
       </c>
       <c r="D9" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="E9">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B10" s="1">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C10" t="s">
         <v>30</v>
       </c>
       <c r="D10" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="E10">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="1" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B11" s="1">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D11" t="s">
         <v>35</v>
       </c>
       <c r="E11">
-        <v>21</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B12" s="1">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D12" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="E12">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B13" s="1">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C13" t="s">
         <v>30</v>
       </c>
       <c r="D13" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="E13">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B14" s="1">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C14" t="s">
         <v>30</v>
       </c>
       <c r="D14" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="E14">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B15" s="1">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C15" t="s">
         <v>34</v>
       </c>
       <c r="D15" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -4303,16 +4322,16 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B16" s="1">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C16" t="s">
         <v>30</v>
       </c>
       <c r="D16" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="E16">
         <v>8</v>
@@ -4320,16 +4339,16 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="1" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B17" s="1">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C17" t="s">
         <v>30</v>
       </c>
       <c r="D17" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="E17">
         <v>15</v>
@@ -4337,41 +4356,92 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B18" s="1">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C18" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="D18" t="s">
-        <v>49</v>
-      </c>
-      <c r="E18" t="s">
-        <v>50</v>
+        <v>44</v>
+      </c>
+      <c r="E18">
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B19" s="1">
+        <v>18</v>
+      </c>
+      <c r="C19" t="s">
+        <v>30</v>
+      </c>
+      <c r="D19" t="s">
+        <v>44</v>
+      </c>
+      <c r="E19">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B20" s="1">
+        <v>19</v>
+      </c>
+      <c r="C20" t="s">
+        <v>30</v>
+      </c>
+      <c r="D20" t="s">
+        <v>44</v>
+      </c>
+      <c r="E20">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B21" s="1">
+        <v>20</v>
+      </c>
+      <c r="C21" t="s">
+        <v>48</v>
+      </c>
+      <c r="D21" t="s">
+        <v>49</v>
+      </c>
+      <c r="E21" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B19" s="1">
+      <c r="B22" s="1">
         <v>21</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C22" t="s">
         <v>34</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D22" t="s">
         <v>52</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E22" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
+    <row r="23" spans="1:5">
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -4382,13 +4452,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="22.58203125" customWidth="1"/>
-    <col min="2" max="2" width="15.08203125" customWidth="1"/>
+    <col min="1" max="1" width="22.5546875" customWidth="1"/>
+    <col min="2" max="2" width="15.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="14.5">
+    <row r="1" spans="1:5" ht="14.4">
       <c r="A1" s="4" t="s">
         <v>145</v>
       </c>

</xml_diff>

<commit_message>
Update cycle_days use type
</commit_message>
<xml_diff>
--- a/inst/extdata/example_visitcode.xlsx
+++ b/inst/extdata/example_visitcode.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="379">
   <si>
     <t>随访期</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1245,6 +1245,10 @@
   </si>
   <si>
     <t>纠正治疗期_D3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CYCDAY</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1615,14 +1619,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="23.6640625" customWidth="1"/>
     <col min="2" max="2" width="18.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="14.4">
+    <row r="1" spans="1:6" ht="14.4">
       <c r="A1" s="4" t="s">
         <v>145</v>
       </c>
@@ -1638,8 +1642,11 @@
       <c r="E1" s="5" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1" s="5" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
         <v>56</v>
       </c>
@@ -1653,7 +1660,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
         <v>57</v>
       </c>
@@ -1667,7 +1674,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
         <v>58</v>
       </c>
@@ -1683,8 +1690,11 @@
       <c r="E4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:5">
+      <c r="F4">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
         <v>59</v>
       </c>
@@ -1700,8 +1710,11 @@
       <c r="E5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:5">
+      <c r="F5">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6" s="1" t="s">
         <v>60</v>
       </c>
@@ -1717,8 +1730,11 @@
       <c r="E6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:5">
+      <c r="F6">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7" s="1" t="s">
         <v>61</v>
       </c>
@@ -1734,8 +1750,11 @@
       <c r="E7">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:5">
+      <c r="F7">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8" s="1" t="s">
         <v>62</v>
       </c>
@@ -1751,8 +1770,11 @@
       <c r="E8">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:5">
+      <c r="F8">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9" s="1" t="s">
         <v>63</v>
       </c>
@@ -1768,8 +1790,11 @@
       <c r="E9">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:5">
+      <c r="F9">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10" s="1" t="s">
         <v>64</v>
       </c>
@@ -1785,8 +1810,11 @@
       <c r="E10">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:5">
+      <c r="F10">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11" s="1" t="s">
         <v>65</v>
       </c>
@@ -1802,8 +1830,11 @@
       <c r="E11">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:5">
+      <c r="F11">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12" s="1" t="s">
         <v>66</v>
       </c>
@@ -1819,8 +1850,11 @@
       <c r="E12">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:5">
+      <c r="F12">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
       <c r="A13" s="1" t="s">
         <v>67</v>
       </c>
@@ -1836,8 +1870,11 @@
       <c r="E13">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:5">
+      <c r="F13">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
       <c r="A14" s="1" t="s">
         <v>68</v>
       </c>
@@ -1853,8 +1890,11 @@
       <c r="E14">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:5">
+      <c r="F14">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
       <c r="A15" s="1" t="s">
         <v>69</v>
       </c>
@@ -1870,8 +1910,11 @@
       <c r="E15">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:5">
+      <c r="F15">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
       <c r="A16" s="1" t="s">
         <v>70</v>
       </c>
@@ -1887,8 +1930,11 @@
       <c r="E16">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:5">
+      <c r="F16">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
       <c r="A17" s="1" t="s">
         <v>71</v>
       </c>
@@ -1904,8 +1950,11 @@
       <c r="E17">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:5">
+      <c r="F17">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
       <c r="A18" s="1" t="s">
         <v>72</v>
       </c>
@@ -1921,8 +1970,11 @@
       <c r="E18">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:5">
+      <c r="F18">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
       <c r="A19" s="1" t="s">
         <v>73</v>
       </c>
@@ -1938,8 +1990,11 @@
       <c r="E19">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:5">
+      <c r="F19">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
       <c r="A20" s="1" t="s">
         <v>74</v>
       </c>
@@ -1955,8 +2010,11 @@
       <c r="E20">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:5">
+      <c r="F20">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
       <c r="A21" s="1" t="s">
         <v>75</v>
       </c>
@@ -1972,8 +2030,11 @@
       <c r="E21">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:5">
+      <c r="F21">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
       <c r="A22" s="1" t="s">
         <v>76</v>
       </c>
@@ -1989,8 +2050,11 @@
       <c r="E22">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:5">
+      <c r="F22">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
       <c r="A23" s="1" t="s">
         <v>77</v>
       </c>
@@ -2006,8 +2070,11 @@
       <c r="E23">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:5">
+      <c r="F23">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
       <c r="A24" s="1" t="s">
         <v>78</v>
       </c>
@@ -2023,8 +2090,11 @@
       <c r="E24">
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:5">
+      <c r="F24">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
       <c r="A25" s="1" t="s">
         <v>79</v>
       </c>
@@ -2040,8 +2110,11 @@
       <c r="E25">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:5">
+      <c r="F25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
       <c r="A26" s="1" t="s">
         <v>80</v>
       </c>
@@ -2057,8 +2130,11 @@
       <c r="E26">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:5">
+      <c r="F26">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
       <c r="A27" s="1" t="s">
         <v>81</v>
       </c>
@@ -2074,8 +2150,11 @@
       <c r="E27">
         <v>1</v>
       </c>
-    </row>
-    <row r="28" spans="1:5">
+      <c r="F27">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
       <c r="A28" s="1" t="s">
         <v>82</v>
       </c>
@@ -2091,8 +2170,11 @@
       <c r="E28">
         <v>1</v>
       </c>
-    </row>
-    <row r="29" spans="1:5">
+      <c r="F28">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
       <c r="A29" s="1" t="s">
         <v>83</v>
       </c>
@@ -2108,8 +2190,11 @@
       <c r="E29">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:5">
+      <c r="F29">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
       <c r="A30" s="1" t="s">
         <v>84</v>
       </c>
@@ -2125,8 +2210,11 @@
       <c r="E30">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="1:5">
+      <c r="F30">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
       <c r="A31" s="1" t="s">
         <v>85</v>
       </c>
@@ -2142,8 +2230,11 @@
       <c r="E31">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:5">
+      <c r="F31">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
       <c r="A32" s="1" t="s">
         <v>86</v>
       </c>
@@ -2159,8 +2250,11 @@
       <c r="E32">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="1:5">
+      <c r="F32">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
       <c r="A33" s="1" t="s">
         <v>87</v>
       </c>
@@ -2176,8 +2270,11 @@
       <c r="E33">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="1:5">
+      <c r="F33">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
       <c r="A34" s="1" t="s">
         <v>88</v>
       </c>
@@ -2193,8 +2290,11 @@
       <c r="E34">
         <v>1</v>
       </c>
-    </row>
-    <row r="35" spans="1:5">
+      <c r="F34">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
       <c r="A35" s="1" t="s">
         <v>89</v>
       </c>
@@ -2210,8 +2310,11 @@
       <c r="E35">
         <v>1</v>
       </c>
-    </row>
-    <row r="36" spans="1:5">
+      <c r="F35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
       <c r="A36" s="1" t="s">
         <v>90</v>
       </c>
@@ -2227,8 +2330,11 @@
       <c r="E36">
         <v>1</v>
       </c>
-    </row>
-    <row r="37" spans="1:5">
+      <c r="F36">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
       <c r="A37" s="1" t="s">
         <v>91</v>
       </c>
@@ -2244,8 +2350,11 @@
       <c r="E37">
         <v>1</v>
       </c>
-    </row>
-    <row r="38" spans="1:5">
+      <c r="F37">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
       <c r="A38" s="1" t="s">
         <v>92</v>
       </c>
@@ -2261,8 +2370,11 @@
       <c r="E38">
         <v>1</v>
       </c>
-    </row>
-    <row r="39" spans="1:5">
+      <c r="F38">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
       <c r="A39" s="1" t="s">
         <v>10</v>
       </c>
@@ -2279,7 +2391,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="40" spans="1:5">
+    <row r="40" spans="1:6">
       <c r="A40" s="1" t="s">
         <v>93</v>
       </c>
@@ -2296,7 +2408,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:6">
       <c r="A41" s="1" t="s">
         <v>94</v>
       </c>
@@ -2313,7 +2425,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:6">
       <c r="A42" s="1" t="s">
         <v>95</v>
       </c>
@@ -2330,7 +2442,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:6">
       <c r="A43" s="1" t="s">
         <v>96</v>
       </c>
@@ -2347,7 +2459,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" spans="1:6">
       <c r="A44" s="1" t="s">
         <v>12</v>
       </c>
@@ -2372,10 +2484,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E99"/>
+  <dimension ref="A1:F99"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>140</v>
       </c>
@@ -2391,8 +2503,11 @@
       <c r="E1" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
         <v>153</v>
       </c>
@@ -2406,7 +2521,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
         <v>157</v>
       </c>
@@ -2423,7 +2538,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
         <v>161</v>
       </c>
@@ -2439,8 +2554,11 @@
       <c r="E4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:5">
+      <c r="F4">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
         <v>164</v>
       </c>
@@ -2456,8 +2574,11 @@
       <c r="E5">
         <v>8</v>
       </c>
-    </row>
-    <row r="6" spans="1:5">
+      <c r="F5">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6" s="1" t="s">
         <v>166</v>
       </c>
@@ -2473,8 +2594,11 @@
       <c r="E6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:5">
+      <c r="F6">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7" s="1" t="s">
         <v>168</v>
       </c>
@@ -2490,8 +2614,11 @@
       <c r="E7">
         <v>8</v>
       </c>
-    </row>
-    <row r="8" spans="1:5">
+      <c r="F7">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8" s="1" t="s">
         <v>170</v>
       </c>
@@ -2507,8 +2634,11 @@
       <c r="E8">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:5">
+      <c r="F8">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9" s="1" t="s">
         <v>172</v>
       </c>
@@ -2524,8 +2654,11 @@
       <c r="E9">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:5">
+      <c r="F9">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10" s="1" t="s">
         <v>175</v>
       </c>
@@ -2541,8 +2674,11 @@
       <c r="E10">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:5">
+      <c r="F10">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11" s="1" t="s">
         <v>177</v>
       </c>
@@ -2558,8 +2694,11 @@
       <c r="E11">
         <v>8</v>
       </c>
-    </row>
-    <row r="12" spans="1:5">
+      <c r="F11">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12" s="1" t="s">
         <v>179</v>
       </c>
@@ -2575,8 +2714,11 @@
       <c r="E12">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:5">
+      <c r="F12">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
       <c r="A13" s="1" t="s">
         <v>181</v>
       </c>
@@ -2592,8 +2734,11 @@
       <c r="E13">
         <v>8</v>
       </c>
-    </row>
-    <row r="14" spans="1:5">
+      <c r="F13">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
       <c r="A14" s="1" t="s">
         <v>183</v>
       </c>
@@ -2609,8 +2754,11 @@
       <c r="E14">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:5">
+      <c r="F14">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
       <c r="A15" s="1" t="s">
         <v>185</v>
       </c>
@@ -2626,8 +2774,11 @@
       <c r="E15">
         <v>8</v>
       </c>
-    </row>
-    <row r="16" spans="1:5">
+      <c r="F15">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
       <c r="A16" s="1" t="s">
         <v>187</v>
       </c>
@@ -2643,8 +2794,11 @@
       <c r="E16">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:5">
+      <c r="F16">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
       <c r="A17" s="1" t="s">
         <v>190</v>
       </c>
@@ -2660,8 +2814,11 @@
       <c r="E17">
         <v>8</v>
       </c>
-    </row>
-    <row r="18" spans="1:5">
+      <c r="F17">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
       <c r="A18" s="1" t="s">
         <v>192</v>
       </c>
@@ -2677,8 +2834,11 @@
       <c r="E18">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:5">
+      <c r="F18">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
       <c r="A19" s="1" t="s">
         <v>194</v>
       </c>
@@ -2694,8 +2854,11 @@
       <c r="E19">
         <v>8</v>
       </c>
-    </row>
-    <row r="20" spans="1:5">
+      <c r="F19">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
       <c r="A20" s="1" t="s">
         <v>196</v>
       </c>
@@ -2711,8 +2874,11 @@
       <c r="E20">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:5">
+      <c r="F20">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
       <c r="A21" s="1" t="s">
         <v>198</v>
       </c>
@@ -2728,8 +2894,11 @@
       <c r="E21">
         <v>8</v>
       </c>
-    </row>
-    <row r="22" spans="1:5">
+      <c r="F21">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
       <c r="A22" s="1" t="s">
         <v>200</v>
       </c>
@@ -2745,8 +2914,11 @@
       <c r="E22">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:5">
+      <c r="F22">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
       <c r="A23" s="1" t="s">
         <v>202</v>
       </c>
@@ -2762,8 +2934,11 @@
       <c r="E23">
         <v>8</v>
       </c>
-    </row>
-    <row r="24" spans="1:5">
+      <c r="F23">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
       <c r="A24" s="1" t="s">
         <v>204</v>
       </c>
@@ -2779,8 +2954,11 @@
       <c r="E24">
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:5">
+      <c r="F24">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
       <c r="A25" s="1" t="s">
         <v>206</v>
       </c>
@@ -2796,8 +2974,11 @@
       <c r="E25">
         <v>8</v>
       </c>
-    </row>
-    <row r="26" spans="1:5">
+      <c r="F25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
       <c r="A26" s="1" t="s">
         <v>208</v>
       </c>
@@ -2813,8 +2994,11 @@
       <c r="E26">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:5">
+      <c r="F26">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
       <c r="A27" s="1" t="s">
         <v>210</v>
       </c>
@@ -2830,8 +3014,11 @@
       <c r="E27">
         <v>8</v>
       </c>
-    </row>
-    <row r="28" spans="1:5">
+      <c r="F27">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
       <c r="A28" s="1" t="s">
         <v>212</v>
       </c>
@@ -2847,8 +3034,11 @@
       <c r="E28">
         <v>1</v>
       </c>
-    </row>
-    <row r="29" spans="1:5">
+      <c r="F28">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
       <c r="A29" s="1" t="s">
         <v>214</v>
       </c>
@@ -2864,8 +3054,11 @@
       <c r="E29">
         <v>8</v>
       </c>
-    </row>
-    <row r="30" spans="1:5">
+      <c r="F29">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
       <c r="A30" s="1" t="s">
         <v>216</v>
       </c>
@@ -2881,8 +3074,11 @@
       <c r="E30">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="1:5">
+      <c r="F30">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
       <c r="A31" s="1" t="s">
         <v>218</v>
       </c>
@@ -2898,8 +3094,11 @@
       <c r="E31">
         <v>8</v>
       </c>
-    </row>
-    <row r="32" spans="1:5">
+      <c r="F31">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
       <c r="A32" s="1" t="s">
         <v>220</v>
       </c>
@@ -2915,8 +3114,11 @@
       <c r="E32">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="1:5">
+      <c r="F32">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
       <c r="A33" s="1" t="s">
         <v>222</v>
       </c>
@@ -2932,8 +3134,11 @@
       <c r="E33">
         <v>8</v>
       </c>
-    </row>
-    <row r="34" spans="1:5">
+      <c r="F33">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
       <c r="A34" s="1" t="s">
         <v>224</v>
       </c>
@@ -2949,8 +3154,11 @@
       <c r="E34">
         <v>1</v>
       </c>
-    </row>
-    <row r="35" spans="1:5">
+      <c r="F34">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
       <c r="A35" s="1" t="s">
         <v>226</v>
       </c>
@@ -2966,8 +3174,11 @@
       <c r="E35">
         <v>8</v>
       </c>
-    </row>
-    <row r="36" spans="1:5">
+      <c r="F35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
       <c r="A36" s="1" t="s">
         <v>228</v>
       </c>
@@ -2983,8 +3194,11 @@
       <c r="E36">
         <v>1</v>
       </c>
-    </row>
-    <row r="37" spans="1:5">
+      <c r="F36">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
       <c r="A37" s="1" t="s">
         <v>230</v>
       </c>
@@ -3000,8 +3214,11 @@
       <c r="E37">
         <v>8</v>
       </c>
-    </row>
-    <row r="38" spans="1:5">
+      <c r="F37">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
       <c r="A38" s="1" t="s">
         <v>232</v>
       </c>
@@ -3017,8 +3234,11 @@
       <c r="E38">
         <v>1</v>
       </c>
-    </row>
-    <row r="39" spans="1:5">
+      <c r="F38">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
       <c r="A39" s="1" t="s">
         <v>234</v>
       </c>
@@ -3034,8 +3254,11 @@
       <c r="E39">
         <v>8</v>
       </c>
-    </row>
-    <row r="40" spans="1:5">
+      <c r="F39">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
       <c r="A40" s="1" t="s">
         <v>236</v>
       </c>
@@ -3051,8 +3274,11 @@
       <c r="E40">
         <v>1</v>
       </c>
-    </row>
-    <row r="41" spans="1:5">
+      <c r="F40">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
       <c r="A41" s="1" t="s">
         <v>238</v>
       </c>
@@ -3068,8 +3294,11 @@
       <c r="E41">
         <v>8</v>
       </c>
-    </row>
-    <row r="42" spans="1:5">
+      <c r="F41">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
       <c r="A42" s="1" t="s">
         <v>240</v>
       </c>
@@ -3085,8 +3314,11 @@
       <c r="E42">
         <v>1</v>
       </c>
-    </row>
-    <row r="43" spans="1:5">
+      <c r="F42">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
       <c r="A43" s="1" t="s">
         <v>242</v>
       </c>
@@ -3102,8 +3334,11 @@
       <c r="E43">
         <v>8</v>
       </c>
-    </row>
-    <row r="44" spans="1:5">
+      <c r="F43">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
       <c r="A44" s="1" t="s">
         <v>244</v>
       </c>
@@ -3119,8 +3354,11 @@
       <c r="E44">
         <v>1</v>
       </c>
-    </row>
-    <row r="45" spans="1:5">
+      <c r="F44">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
       <c r="A45" s="1" t="s">
         <v>246</v>
       </c>
@@ -3136,8 +3374,11 @@
       <c r="E45">
         <v>8</v>
       </c>
-    </row>
-    <row r="46" spans="1:5">
+      <c r="F45">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6">
       <c r="A46" s="1" t="s">
         <v>248</v>
       </c>
@@ -3153,8 +3394,11 @@
       <c r="E46">
         <v>1</v>
       </c>
-    </row>
-    <row r="47" spans="1:5">
+      <c r="F46">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
       <c r="A47" s="1" t="s">
         <v>250</v>
       </c>
@@ -3170,8 +3414,11 @@
       <c r="E47">
         <v>8</v>
       </c>
-    </row>
-    <row r="48" spans="1:5">
+      <c r="F47">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6">
       <c r="A48" s="1" t="s">
         <v>252</v>
       </c>
@@ -3187,8 +3434,11 @@
       <c r="E48">
         <v>1</v>
       </c>
-    </row>
-    <row r="49" spans="1:5">
+      <c r="F48">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
       <c r="A49" s="1" t="s">
         <v>254</v>
       </c>
@@ -3204,8 +3454,11 @@
       <c r="E49">
         <v>8</v>
       </c>
-    </row>
-    <row r="50" spans="1:5">
+      <c r="F49">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
       <c r="A50" s="1" t="s">
         <v>256</v>
       </c>
@@ -3221,8 +3474,11 @@
       <c r="E50">
         <v>1</v>
       </c>
-    </row>
-    <row r="51" spans="1:5">
+      <c r="F50">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
       <c r="A51" s="1" t="s">
         <v>258</v>
       </c>
@@ -3238,8 +3494,11 @@
       <c r="E51">
         <v>8</v>
       </c>
-    </row>
-    <row r="52" spans="1:5">
+      <c r="F51">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
       <c r="A52" s="1" t="s">
         <v>260</v>
       </c>
@@ -3255,8 +3514,11 @@
       <c r="E52">
         <v>1</v>
       </c>
-    </row>
-    <row r="53" spans="1:5">
+      <c r="F52">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6">
       <c r="A53" s="1" t="s">
         <v>262</v>
       </c>
@@ -3272,8 +3534,11 @@
       <c r="E53">
         <v>8</v>
       </c>
-    </row>
-    <row r="54" spans="1:5">
+      <c r="F53">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6">
       <c r="A54" s="1" t="s">
         <v>264</v>
       </c>
@@ -3289,8 +3554,11 @@
       <c r="E54">
         <v>1</v>
       </c>
-    </row>
-    <row r="55" spans="1:5">
+      <c r="F54">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6">
       <c r="A55" s="1" t="s">
         <v>266</v>
       </c>
@@ -3306,8 +3574,11 @@
       <c r="E55">
         <v>8</v>
       </c>
-    </row>
-    <row r="56" spans="1:5">
+      <c r="F55">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6">
       <c r="A56" s="1" t="s">
         <v>268</v>
       </c>
@@ -3323,8 +3594,11 @@
       <c r="E56">
         <v>1</v>
       </c>
-    </row>
-    <row r="57" spans="1:5">
+      <c r="F56">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6">
       <c r="A57" s="1" t="s">
         <v>270</v>
       </c>
@@ -3340,8 +3614,11 @@
       <c r="E57">
         <v>8</v>
       </c>
-    </row>
-    <row r="58" spans="1:5">
+      <c r="F57">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6">
       <c r="A58" s="1" t="s">
         <v>272</v>
       </c>
@@ -3357,8 +3634,11 @@
       <c r="E58">
         <v>1</v>
       </c>
-    </row>
-    <row r="59" spans="1:5">
+      <c r="F58">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6">
       <c r="A59" s="1" t="s">
         <v>274</v>
       </c>
@@ -3374,8 +3654,11 @@
       <c r="E59">
         <v>8</v>
       </c>
-    </row>
-    <row r="60" spans="1:5">
+      <c r="F59">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
       <c r="A60" s="1" t="s">
         <v>276</v>
       </c>
@@ -3391,8 +3674,11 @@
       <c r="E60">
         <v>1</v>
       </c>
-    </row>
-    <row r="61" spans="1:5">
+      <c r="F60">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
       <c r="A61" s="1" t="s">
         <v>278</v>
       </c>
@@ -3408,8 +3694,11 @@
       <c r="E61">
         <v>8</v>
       </c>
-    </row>
-    <row r="62" spans="1:5">
+      <c r="F61">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
       <c r="A62" s="1" t="s">
         <v>280</v>
       </c>
@@ -3425,8 +3714,11 @@
       <c r="E62">
         <v>1</v>
       </c>
-    </row>
-    <row r="63" spans="1:5">
+      <c r="F62">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
       <c r="A63" s="1" t="s">
         <v>282</v>
       </c>
@@ -3442,8 +3734,11 @@
       <c r="E63">
         <v>8</v>
       </c>
-    </row>
-    <row r="64" spans="1:5">
+      <c r="F63">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6">
       <c r="A64" s="1" t="s">
         <v>284</v>
       </c>
@@ -3459,8 +3754,11 @@
       <c r="E64">
         <v>1</v>
       </c>
-    </row>
-    <row r="65" spans="1:5">
+      <c r="F64">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6">
       <c r="A65" s="1" t="s">
         <v>286</v>
       </c>
@@ -3476,8 +3774,11 @@
       <c r="E65">
         <v>8</v>
       </c>
-    </row>
-    <row r="66" spans="1:5">
+      <c r="F65">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6">
       <c r="A66" s="1" t="s">
         <v>288</v>
       </c>
@@ -3493,8 +3794,11 @@
       <c r="E66">
         <v>1</v>
       </c>
-    </row>
-    <row r="67" spans="1:5">
+      <c r="F66">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6">
       <c r="A67" s="1" t="s">
         <v>290</v>
       </c>
@@ -3510,8 +3814,11 @@
       <c r="E67">
         <v>8</v>
       </c>
-    </row>
-    <row r="68" spans="1:5">
+      <c r="F67">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6">
       <c r="A68" s="1" t="s">
         <v>292</v>
       </c>
@@ -3527,8 +3834,11 @@
       <c r="E68">
         <v>1</v>
       </c>
-    </row>
-    <row r="69" spans="1:5">
+      <c r="F68">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6">
       <c r="A69" s="1" t="s">
         <v>294</v>
       </c>
@@ -3544,8 +3854,11 @@
       <c r="E69">
         <v>8</v>
       </c>
-    </row>
-    <row r="70" spans="1:5">
+      <c r="F69">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6">
       <c r="A70" s="1" t="s">
         <v>296</v>
       </c>
@@ -3561,8 +3874,11 @@
       <c r="E70">
         <v>1</v>
       </c>
-    </row>
-    <row r="71" spans="1:5">
+      <c r="F70">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6">
       <c r="A71" s="1" t="s">
         <v>298</v>
       </c>
@@ -3578,8 +3894,11 @@
       <c r="E71">
         <v>8</v>
       </c>
-    </row>
-    <row r="72" spans="1:5">
+      <c r="F71">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6">
       <c r="A72" s="1" t="s">
         <v>300</v>
       </c>
@@ -3595,8 +3914,11 @@
       <c r="E72">
         <v>1</v>
       </c>
-    </row>
-    <row r="73" spans="1:5">
+      <c r="F72">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6">
       <c r="A73" s="1" t="s">
         <v>302</v>
       </c>
@@ -3612,8 +3934,11 @@
       <c r="E73">
         <v>8</v>
       </c>
-    </row>
-    <row r="74" spans="1:5">
+      <c r="F73">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6">
       <c r="A74" s="1" t="s">
         <v>304</v>
       </c>
@@ -3629,8 +3954,11 @@
       <c r="E74">
         <v>1</v>
       </c>
-    </row>
-    <row r="75" spans="1:5">
+      <c r="F74">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6">
       <c r="A75" s="1" t="s">
         <v>307</v>
       </c>
@@ -3646,8 +3974,11 @@
       <c r="E75">
         <v>8</v>
       </c>
-    </row>
-    <row r="76" spans="1:5">
+      <c r="F75">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6">
       <c r="A76" s="1" t="s">
         <v>309</v>
       </c>
@@ -3663,8 +3994,11 @@
       <c r="E76">
         <v>1</v>
       </c>
-    </row>
-    <row r="77" spans="1:5">
+      <c r="F76">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6">
       <c r="A77" s="1" t="s">
         <v>312</v>
       </c>
@@ -3680,8 +4014,11 @@
       <c r="E77">
         <v>8</v>
       </c>
-    </row>
-    <row r="78" spans="1:5">
+      <c r="F77">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6">
       <c r="A78" s="1" t="s">
         <v>314</v>
       </c>
@@ -3697,8 +4034,11 @@
       <c r="E78">
         <v>1</v>
       </c>
-    </row>
-    <row r="79" spans="1:5">
+      <c r="F78">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6">
       <c r="A79" s="1" t="s">
         <v>317</v>
       </c>
@@ -3714,8 +4054,11 @@
       <c r="E79">
         <v>8</v>
       </c>
-    </row>
-    <row r="80" spans="1:5">
+      <c r="F79">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6">
       <c r="A80" s="1" t="s">
         <v>319</v>
       </c>
@@ -3731,8 +4074,11 @@
       <c r="E80">
         <v>1</v>
       </c>
-    </row>
-    <row r="81" spans="1:5">
+      <c r="F80">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6">
       <c r="A81" s="1" t="s">
         <v>322</v>
       </c>
@@ -3748,8 +4094,11 @@
       <c r="E81">
         <v>8</v>
       </c>
-    </row>
-    <row r="82" spans="1:5">
+      <c r="F81">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6">
       <c r="A82" s="1" t="s">
         <v>324</v>
       </c>
@@ -3765,8 +4114,11 @@
       <c r="E82">
         <v>1</v>
       </c>
-    </row>
-    <row r="83" spans="1:5">
+      <c r="F82">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6">
       <c r="A83" s="1" t="s">
         <v>327</v>
       </c>
@@ -3782,8 +4134,11 @@
       <c r="E83">
         <v>8</v>
       </c>
-    </row>
-    <row r="84" spans="1:5">
+      <c r="F83">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6">
       <c r="A84" s="1" t="s">
         <v>329</v>
       </c>
@@ -3799,8 +4154,11 @@
       <c r="E84">
         <v>1</v>
       </c>
-    </row>
-    <row r="85" spans="1:5">
+      <c r="F84">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6">
       <c r="A85" s="1" t="s">
         <v>332</v>
       </c>
@@ -3816,8 +4174,11 @@
       <c r="E85">
         <v>8</v>
       </c>
-    </row>
-    <row r="86" spans="1:5">
+      <c r="F85">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6">
       <c r="A86" s="1" t="s">
         <v>334</v>
       </c>
@@ -3833,8 +4194,11 @@
       <c r="E86">
         <v>1</v>
       </c>
-    </row>
-    <row r="87" spans="1:5">
+      <c r="F86">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6">
       <c r="A87" s="1" t="s">
         <v>337</v>
       </c>
@@ -3850,8 +4214,11 @@
       <c r="E87">
         <v>8</v>
       </c>
-    </row>
-    <row r="88" spans="1:5">
+      <c r="F87">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6">
       <c r="A88" s="1" t="s">
         <v>339</v>
       </c>
@@ -3867,8 +4234,11 @@
       <c r="E88">
         <v>1</v>
       </c>
-    </row>
-    <row r="89" spans="1:5">
+      <c r="F88">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6">
       <c r="A89" s="1" t="s">
         <v>342</v>
       </c>
@@ -3884,8 +4254,11 @@
       <c r="E89">
         <v>8</v>
       </c>
-    </row>
-    <row r="90" spans="1:5">
+      <c r="F89">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6">
       <c r="A90" s="1" t="s">
         <v>344</v>
       </c>
@@ -3901,8 +4274,11 @@
       <c r="E90">
         <v>1</v>
       </c>
-    </row>
-    <row r="91" spans="1:5">
+      <c r="F90">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6">
       <c r="A91" s="1" t="s">
         <v>347</v>
       </c>
@@ -3918,8 +4294,11 @@
       <c r="E91">
         <v>8</v>
       </c>
-    </row>
-    <row r="92" spans="1:5">
+      <c r="F91">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6">
       <c r="A92" s="1" t="s">
         <v>349</v>
       </c>
@@ -3935,8 +4314,11 @@
       <c r="E92">
         <v>1</v>
       </c>
-    </row>
-    <row r="93" spans="1:5">
+      <c r="F92">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6">
       <c r="A93" s="1" t="s">
         <v>352</v>
       </c>
@@ -3952,8 +4334,11 @@
       <c r="E93">
         <v>8</v>
       </c>
-    </row>
-    <row r="94" spans="1:5">
+      <c r="F93">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6">
       <c r="A94" s="1" t="s">
         <v>354</v>
       </c>
@@ -3970,7 +4355,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="95" spans="1:5">
+    <row r="95" spans="1:6">
       <c r="A95" s="1" t="s">
         <v>359</v>
       </c>
@@ -3987,7 +4372,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="96" spans="1:5">
+    <row r="96" spans="1:6">
       <c r="A96" s="1" t="s">
         <v>361</v>
       </c>
@@ -4063,7 +4448,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="21.6640625" customWidth="1"/>
@@ -4071,7 +4456,7 @@
     <col min="3" max="3" width="9.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="14.4">
+    <row r="1" spans="1:6" ht="14.4">
       <c r="A1" s="4" t="s">
         <v>140</v>
       </c>
@@ -4087,8 +4472,11 @@
       <c r="E1" s="5" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1" s="5" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
         <v>21</v>
       </c>
@@ -4102,7 +4490,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
         <v>24</v>
       </c>
@@ -4116,7 +4504,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:6">
       <c r="A4" s="10" t="s">
         <v>374</v>
       </c>
@@ -4133,7 +4521,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:6">
       <c r="A5" s="10" t="s">
         <v>376</v>
       </c>
@@ -4150,7 +4538,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:6">
       <c r="A6" s="10" t="s">
         <v>377</v>
       </c>
@@ -4167,7 +4555,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:6">
       <c r="A7" s="1" t="s">
         <v>27</v>
       </c>
@@ -4183,8 +4571,11 @@
       <c r="E7">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:5">
+      <c r="F7">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8" s="1" t="s">
         <v>29</v>
       </c>
@@ -4200,8 +4591,11 @@
       <c r="E8">
         <v>8</v>
       </c>
-    </row>
-    <row r="9" spans="1:5">
+      <c r="F8">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9" s="1" t="s">
         <v>31</v>
       </c>
@@ -4217,8 +4611,11 @@
       <c r="E9">
         <v>15</v>
       </c>
-    </row>
-    <row r="10" spans="1:5">
+      <c r="F9">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10" s="1" t="s">
         <v>32</v>
       </c>
@@ -4234,8 +4631,11 @@
       <c r="E10">
         <v>21</v>
       </c>
-    </row>
-    <row r="11" spans="1:5">
+      <c r="F10">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11" s="1" t="s">
         <v>33</v>
       </c>
@@ -4251,8 +4651,11 @@
       <c r="E11">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:5">
+      <c r="F11">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12" s="1" t="s">
         <v>36</v>
       </c>
@@ -4268,8 +4671,11 @@
       <c r="E12">
         <v>8</v>
       </c>
-    </row>
-    <row r="13" spans="1:5">
+      <c r="F12">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
       <c r="A13" s="1" t="s">
         <v>37</v>
       </c>
@@ -4285,8 +4691,11 @@
       <c r="E13">
         <v>15</v>
       </c>
-    </row>
-    <row r="14" spans="1:5">
+      <c r="F13">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
       <c r="A14" s="1" t="s">
         <v>38</v>
       </c>
@@ -4302,8 +4711,11 @@
       <c r="E14">
         <v>21</v>
       </c>
-    </row>
-    <row r="15" spans="1:5">
+      <c r="F14">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
       <c r="A15" s="1" t="s">
         <v>39</v>
       </c>
@@ -4319,8 +4731,11 @@
       <c r="E15">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:5">
+      <c r="F15">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
       <c r="A16" s="1" t="s">
         <v>41</v>
       </c>
@@ -4336,8 +4751,11 @@
       <c r="E16">
         <v>8</v>
       </c>
-    </row>
-    <row r="17" spans="1:5">
+      <c r="F16">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
       <c r="A17" s="1" t="s">
         <v>42</v>
       </c>
@@ -4353,8 +4771,11 @@
       <c r="E17">
         <v>15</v>
       </c>
-    </row>
-    <row r="18" spans="1:5">
+      <c r="F17">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
       <c r="A18" s="1" t="s">
         <v>43</v>
       </c>
@@ -4370,8 +4791,11 @@
       <c r="E18">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:5">
+      <c r="F18">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
       <c r="A19" s="1" t="s">
         <v>45</v>
       </c>
@@ -4387,8 +4811,11 @@
       <c r="E19">
         <v>8</v>
       </c>
-    </row>
-    <row r="20" spans="1:5">
+      <c r="F19">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
       <c r="A20" s="1" t="s">
         <v>46</v>
       </c>
@@ -4404,8 +4831,11 @@
       <c r="E20">
         <v>15</v>
       </c>
-    </row>
-    <row r="21" spans="1:5">
+      <c r="F20">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
       <c r="A21" s="1" t="s">
         <v>47</v>
       </c>
@@ -4422,7 +4852,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:6">
       <c r="A22" s="1" t="s">
         <v>51</v>
       </c>
@@ -4439,7 +4869,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:6">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
     </row>

</xml_diff>